<commit_message>
commit: fixed gantt chart
</commit_message>
<xml_diff>
--- a/Documents/Gantt Chart.xlsx
+++ b/Documents/Gantt Chart.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Jerry\Documents\GitHub\Honours-Project-PCG-of-3D-Platformers-\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCC11199-18EE-480E-A766-A9E712353C67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95219DAA-EE12-42A7-8F9F-FD057ED65CBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{1119FB18-55D4-4D97-9D7D-B7A1FA1BF5AA}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="89">
   <si>
     <t>Task</t>
   </si>
@@ -47,12 +47,6 @@
     <t>End Date</t>
   </si>
   <si>
-    <t>Days</t>
-  </si>
-  <si>
-    <t>Progress</t>
-  </si>
-  <si>
     <t>Implementation</t>
   </si>
   <si>
@@ -113,14 +107,209 @@
     <t>Project Demo Preparation</t>
   </si>
   <si>
-    <t>01/19/26</t>
+    <t>Implementing a PCG Level Prototype</t>
+  </si>
+  <si>
+    <t>Platform Mesh Design (Started 28/10/25)</t>
+  </si>
+  <si>
+    <t>Platforms requiring jumping up/down</t>
+  </si>
+  <si>
+    <t>Player character</t>
+  </si>
+  <si>
+    <t>Generating platforms based on state</t>
+  </si>
+  <si>
+    <t>Generating list of states (rather than predefined)</t>
+  </si>
+  <si>
+    <t>Direction Change % chance (can be adjusted in engine)</t>
+  </si>
+  <si>
+    <t>Angles between two platforms (rather than four directions)</t>
+  </si>
+  <si>
+    <t>Procedural placement of collectables and static objects</t>
+  </si>
+  <si>
+    <t>Introduction</t>
+  </si>
+  <si>
+    <t>Literature Review</t>
+  </si>
+  <si>
+    <t>Methodology</t>
+  </si>
+  <si>
+    <t>Results</t>
+  </si>
+  <si>
+    <t>Discussion</t>
+  </si>
+  <si>
+    <t>Conclusion and Future Work</t>
+  </si>
+  <si>
+    <t>Final Touches</t>
+  </si>
+  <si>
+    <t>Hand-In</t>
+  </si>
+  <si>
+    <t>Project Hand-In</t>
+  </si>
+  <si>
+    <t>Dissertation Hand-In</t>
+  </si>
+  <si>
+    <t>Ethics/Risk Assessment</t>
+  </si>
+  <si>
+    <t>Research on PCG and Level Design (For Feasibility Demo)</t>
+  </si>
+  <si>
+    <t>Feasibility Demo Preparation</t>
+  </si>
+  <si>
+    <t>Developing Lit Review/Annotated Bibliography</t>
+  </si>
+  <si>
+    <t>Survey Design</t>
+  </si>
+  <si>
+    <t>Risk Analysis</t>
+  </si>
+  <si>
+    <t>Feasability Demo Hand-In</t>
+  </si>
+  <si>
+    <t>Duration</t>
+  </si>
+  <si>
+    <t>Week Beginning:</t>
+  </si>
+  <si>
+    <t>S1 Week 9</t>
+  </si>
+  <si>
+    <t>S1 Week 8</t>
+  </si>
+  <si>
+    <t>S1 Week 10</t>
+  </si>
+  <si>
+    <t>S1 Week 11</t>
+  </si>
+  <si>
+    <t>S1 Week 12</t>
+  </si>
+  <si>
+    <t>S2 Week 1</t>
+  </si>
+  <si>
+    <t>S2 Week 2</t>
+  </si>
+  <si>
+    <t>S2 Week 3</t>
+  </si>
+  <si>
+    <t>S2 Week 4</t>
+  </si>
+  <si>
+    <t>S2 Week 5</t>
+  </si>
+  <si>
+    <t>S2 Week 6</t>
+  </si>
+  <si>
+    <t>S2 Week 7</t>
+  </si>
+  <si>
+    <t>S2 Week 8</t>
+  </si>
+  <si>
+    <t>S2 Week 9</t>
+  </si>
+  <si>
+    <t>S2 Week 10</t>
+  </si>
+  <si>
+    <t>Spring Break 1</t>
+  </si>
+  <si>
+    <t>Spring Break 2</t>
+  </si>
+  <si>
+    <t>S2 Week 11</t>
+  </si>
+  <si>
+    <t>S2 Week 12</t>
+  </si>
+  <si>
+    <t>S2 Week 13</t>
+  </si>
+  <si>
+    <t>S2 Week 14</t>
+  </si>
+  <si>
+    <t>End</t>
+  </si>
+  <si>
+    <t>Week:</t>
+  </si>
+  <si>
+    <t>6 days</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23 days </t>
+  </si>
+  <si>
+    <t>22 days</t>
+  </si>
+  <si>
+    <t>15 days</t>
+  </si>
+  <si>
+    <t>7 days</t>
+  </si>
+  <si>
+    <t>1 day</t>
+  </si>
+  <si>
+    <t>46 days</t>
+  </si>
+  <si>
+    <t>8 days</t>
+  </si>
+  <si>
+    <t>5 days</t>
+  </si>
+  <si>
+    <t>2 days</t>
+  </si>
+  <si>
+    <t>3 days</t>
+  </si>
+  <si>
+    <t>57 days</t>
+  </si>
+  <si>
+    <t>73 days</t>
+  </si>
+  <si>
+    <t>26 days</t>
+  </si>
+  <si>
+    <t>Player Character Model, Animations, and Refinement</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -136,13 +325,86 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="9" tint="-0.249977111117893"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0070C0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -157,13 +419,30 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -498,158 +777,910 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C63CAE2-8401-49FA-BE9B-32E21946B78F}">
-  <dimension ref="A8:E38"/>
+  <dimension ref="A7:AB64"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="56.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="11" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="17" max="18" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="22" max="23" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="24" max="28" width="10.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="F7" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G7" t="s">
+        <v>52</v>
+      </c>
+      <c r="H7" t="s">
+        <v>51</v>
+      </c>
+      <c r="I7" t="s">
+        <v>53</v>
+      </c>
+      <c r="J7" t="s">
+        <v>54</v>
+      </c>
+      <c r="K7" t="s">
+        <v>55</v>
+      </c>
+      <c r="L7" t="s">
+        <v>56</v>
+      </c>
+      <c r="M7" t="s">
+        <v>57</v>
+      </c>
+      <c r="N7" t="s">
+        <v>58</v>
+      </c>
+      <c r="O7" t="s">
+        <v>59</v>
+      </c>
+      <c r="P7" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>61</v>
+      </c>
+      <c r="R7" t="s">
+        <v>62</v>
+      </c>
+      <c r="S7" t="s">
+        <v>63</v>
+      </c>
+      <c r="T7" t="s">
+        <v>64</v>
+      </c>
+      <c r="U7" t="s">
+        <v>65</v>
+      </c>
+      <c r="V7" t="s">
+        <v>66</v>
+      </c>
+      <c r="W7" t="s">
+        <v>67</v>
+      </c>
+      <c r="X7" t="s">
+        <v>68</v>
+      </c>
+      <c r="Y7" t="s">
+        <v>69</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>70</v>
+      </c>
+      <c r="AA7" t="s">
+        <v>71</v>
+      </c>
+      <c r="AB7" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G8" s="2">
+        <v>45964</v>
+      </c>
+      <c r="H8" s="2">
+        <v>45971</v>
+      </c>
+      <c r="I8" s="2">
+        <v>45978</v>
+      </c>
+      <c r="J8" s="2">
+        <v>45985</v>
+      </c>
+      <c r="K8" s="2">
+        <v>45992</v>
+      </c>
+      <c r="L8" s="2">
+        <v>46041</v>
+      </c>
+      <c r="M8" s="2">
+        <v>46048</v>
+      </c>
+      <c r="N8" s="2">
+        <v>46055</v>
+      </c>
+      <c r="O8" s="2">
+        <v>46062</v>
+      </c>
+      <c r="P8" s="2">
+        <v>46069</v>
+      </c>
+      <c r="Q8" s="2">
+        <v>46076</v>
+      </c>
+      <c r="R8" s="2">
+        <v>46083</v>
+      </c>
+      <c r="S8" s="2">
+        <v>46090</v>
+      </c>
+      <c r="T8" s="2">
+        <v>46097</v>
+      </c>
+      <c r="U8" s="2">
+        <v>46104</v>
+      </c>
+      <c r="V8" s="2">
+        <v>46111</v>
+      </c>
+      <c r="W8" s="2">
+        <v>46118</v>
+      </c>
+      <c r="X8" s="2">
+        <v>46125</v>
+      </c>
+      <c r="Y8" s="2">
+        <v>46132</v>
+      </c>
+      <c r="Z8" s="2">
+        <v>46139</v>
+      </c>
+      <c r="AA8" s="2">
+        <v>46146</v>
+      </c>
+      <c r="AB8" s="2">
+        <v>46153</v>
+      </c>
+    </row>
+    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" s="2">
+        <v>45964</v>
+      </c>
+      <c r="C10" s="2">
+        <v>45987</v>
+      </c>
+      <c r="D10" t="s">
+        <v>75</v>
+      </c>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
+      <c r="K10" s="8"/>
+    </row>
+    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" s="2">
+        <v>45964</v>
+      </c>
+      <c r="C11" s="2">
+        <v>45986</v>
+      </c>
+      <c r="D11" t="s">
+        <v>76</v>
+      </c>
+      <c r="G11" s="6"/>
+      <c r="H11" s="6"/>
+      <c r="I11" s="6"/>
+      <c r="J11" s="6"/>
+      <c r="K11" s="6"/>
+    </row>
+    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B12" s="2">
+        <v>45964</v>
+      </c>
+      <c r="C12" s="2">
+        <v>45964</v>
+      </c>
+      <c r="D12" t="s">
+        <v>79</v>
+      </c>
+      <c r="G12" s="7"/>
+    </row>
+    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13" s="2">
+        <v>45984</v>
+      </c>
+      <c r="C13" s="2">
+        <v>45986</v>
+      </c>
+      <c r="D13" t="s">
+        <v>84</v>
+      </c>
+      <c r="J13" s="7"/>
+    </row>
+    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="2">
+        <v>45966</v>
+      </c>
+      <c r="C14" s="2">
+        <v>45968</v>
+      </c>
+      <c r="D14" t="s">
+        <v>84</v>
+      </c>
+      <c r="G14" s="7"/>
+    </row>
+    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" s="2">
+        <v>45964</v>
+      </c>
+      <c r="C15" s="2">
+        <v>45966</v>
+      </c>
+      <c r="D15" t="s">
+        <v>84</v>
+      </c>
+      <c r="G15" s="7"/>
+    </row>
+    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B16" s="2">
+        <v>45986</v>
+      </c>
+      <c r="C16" s="2">
+        <v>45986</v>
+      </c>
+      <c r="D16" t="s">
+        <v>79</v>
+      </c>
+      <c r="J16" s="7"/>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B17" s="2">
+        <v>45986</v>
+      </c>
+      <c r="C17" s="2">
+        <v>45986</v>
+      </c>
+      <c r="D17" t="s">
+        <v>79</v>
+      </c>
+      <c r="J17" s="7"/>
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B18" s="2">
+        <v>45971</v>
+      </c>
+      <c r="C18" s="2">
+        <v>46342</v>
+      </c>
+      <c r="D18" t="s">
+        <v>74</v>
+      </c>
+      <c r="H18" s="16"/>
+    </row>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B19" s="2">
+        <v>45969</v>
+      </c>
+      <c r="C19" s="2">
+        <v>45983</v>
+      </c>
+      <c r="D19" t="s">
+        <v>77</v>
+      </c>
+      <c r="G19" s="15"/>
+      <c r="H19" s="15"/>
+      <c r="I19" s="15"/>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B20" s="2">
+        <v>45979</v>
+      </c>
+      <c r="C20" s="2">
+        <v>45986</v>
+      </c>
+      <c r="D20" t="s">
+        <v>78</v>
+      </c>
+      <c r="I20" s="5"/>
+      <c r="J20" s="5"/>
+    </row>
+    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B21" s="2">
+        <v>45976</v>
+      </c>
+      <c r="C21" s="2">
+        <v>45977</v>
+      </c>
+      <c r="D21" t="s">
+        <v>83</v>
+      </c>
+      <c r="I21" s="5"/>
+    </row>
+    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B22" s="2">
+        <v>45976</v>
+      </c>
+      <c r="C22" s="2">
+        <v>45980</v>
+      </c>
+      <c r="D22" t="s">
+        <v>82</v>
+      </c>
+      <c r="I22" s="5"/>
+    </row>
+    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B23" s="2">
+        <v>45987</v>
+      </c>
+      <c r="C23" s="2">
+        <v>45987</v>
+      </c>
+      <c r="D23" t="s">
+        <v>79</v>
+      </c>
+      <c r="J23" s="11"/>
+    </row>
+    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E8" t="s">
+      <c r="B25" s="2">
+        <v>46041</v>
+      </c>
+      <c r="C25" s="2">
+        <v>46086</v>
+      </c>
+      <c r="D25" t="s">
+        <v>80</v>
+      </c>
+      <c r="L25" s="8"/>
+      <c r="M25" s="8"/>
+      <c r="N25" s="8"/>
+      <c r="O25" s="8"/>
+      <c r="P25" s="8"/>
+      <c r="Q25" s="8"/>
+      <c r="R25" s="8"/>
+      <c r="S25" s="14"/>
+    </row>
+    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+      <c r="B26" s="2">
+        <v>46041</v>
+      </c>
+      <c r="C26" s="2">
+        <v>46047</v>
+      </c>
+      <c r="D26" t="s">
+        <v>78</v>
+      </c>
+      <c r="L26" s="7"/>
+    </row>
+    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
+      <c r="B27" s="2">
+        <v>46048</v>
+      </c>
+      <c r="C27" s="2">
+        <v>46055</v>
+      </c>
+      <c r="D27" t="s">
+        <v>81</v>
+      </c>
+      <c r="M27" s="7"/>
+    </row>
+    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B28" s="2">
+        <v>46055</v>
+      </c>
+      <c r="C28" s="2">
+        <v>46205</v>
+      </c>
+      <c r="D28" t="s">
+        <v>82</v>
+      </c>
+      <c r="N28" s="7"/>
+    </row>
+    <row r="29" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B11" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
+      <c r="B29" s="2">
+        <v>46056</v>
+      </c>
+      <c r="C29" s="2">
+        <v>45697</v>
+      </c>
+      <c r="D29" t="s">
+        <v>78</v>
+      </c>
+      <c r="N29" s="7"/>
+    </row>
+    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
+      <c r="B30" s="2">
+        <v>46063</v>
+      </c>
+      <c r="C30" s="2">
+        <v>46070</v>
+      </c>
+      <c r="D30" t="s">
+        <v>81</v>
+      </c>
+      <c r="O30" s="7"/>
+      <c r="P30" s="7"/>
+    </row>
+    <row r="31" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2">
+        <v>46071</v>
+      </c>
+      <c r="C31" s="2">
+        <v>46078</v>
+      </c>
+      <c r="D31" t="s">
+        <v>81</v>
+      </c>
+      <c r="P31" s="7"/>
+      <c r="Q31" s="7"/>
+      <c r="S31" s="14"/>
+    </row>
+    <row r="32" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A32" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2">
+        <v>46079</v>
+      </c>
+      <c r="C32" s="2">
+        <v>46086</v>
+      </c>
+      <c r="D32" t="s">
+        <v>81</v>
+      </c>
+      <c r="Q32" s="7"/>
+      <c r="R32" s="7"/>
+    </row>
+    <row r="34" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
+      <c r="B34" s="2">
+        <v>46079</v>
+      </c>
+      <c r="C34" s="2">
+        <v>46104</v>
+      </c>
+      <c r="D34" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q34" s="8"/>
+      <c r="R34" s="8"/>
+      <c r="S34" s="8"/>
+      <c r="T34" s="8"/>
+      <c r="U34" s="14"/>
+    </row>
+    <row r="35" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A35" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
+      <c r="B35" s="2">
+        <v>46079</v>
+      </c>
+      <c r="C35" s="2">
+        <v>46086</v>
+      </c>
+      <c r="D35" t="s">
+        <v>81</v>
+      </c>
+      <c r="Q35" s="13"/>
+      <c r="R35" s="13"/>
+    </row>
+    <row r="36" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A36" s="3" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
+      <c r="B36" s="2">
+        <v>46083</v>
+      </c>
+      <c r="C36" s="2">
+        <v>46089</v>
+      </c>
+      <c r="D36" t="s">
+        <v>78</v>
+      </c>
+      <c r="R36" s="13"/>
+    </row>
+    <row r="37" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A37" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
+      <c r="B37" s="2">
+        <v>46090</v>
+      </c>
+      <c r="C37" s="2">
+        <v>46097</v>
+      </c>
+      <c r="D37" t="s">
+        <v>81</v>
+      </c>
+      <c r="R37" s="14"/>
+      <c r="S37" s="13"/>
+    </row>
+    <row r="38" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A38" s="3" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
+      <c r="B38" s="2">
+        <v>46097</v>
+      </c>
+      <c r="C38" s="2">
+        <v>46104</v>
+      </c>
+      <c r="D38" t="s">
+        <v>81</v>
+      </c>
+      <c r="S38" s="14"/>
+      <c r="T38" s="13"/>
+    </row>
+    <row r="40" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A40" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
+    <row r="41" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A41" s="3" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
+      <c r="B41" s="2">
+        <v>46041</v>
+      </c>
+      <c r="C41" s="2">
+        <v>46097</v>
+      </c>
+      <c r="D41" t="s">
+        <v>85</v>
+      </c>
+      <c r="M41" s="5"/>
+      <c r="N41" s="5"/>
+      <c r="O41" s="5"/>
+      <c r="P41" s="5"/>
+      <c r="Q41" s="5"/>
+      <c r="R41" s="5"/>
+      <c r="S41" s="5"/>
+      <c r="T41" s="14"/>
+    </row>
+    <row r="43" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A43" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" s="3" t="s">
+    <row r="44" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A44" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B44" s="2">
+        <v>46083</v>
+      </c>
+      <c r="C44" s="2">
+        <v>46090</v>
+      </c>
+      <c r="D44" t="s">
+        <v>81</v>
+      </c>
+      <c r="R44" s="9"/>
+    </row>
+    <row r="45" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A45" s="3" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" s="3" t="s">
+      <c r="B45" s="2">
+        <v>46097</v>
+      </c>
+      <c r="C45" s="2">
+        <v>46104</v>
+      </c>
+      <c r="D45" t="s">
+        <v>81</v>
+      </c>
+      <c r="T45" s="9"/>
+    </row>
+    <row r="46" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A46" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B46" s="2">
+        <v>46104</v>
+      </c>
+      <c r="C46" s="2">
+        <v>46108</v>
+      </c>
+      <c r="D46" t="s">
+        <v>82</v>
+      </c>
+      <c r="U46" s="9"/>
+    </row>
+    <row r="47" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A47" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B27" s="2">
+      <c r="B47" s="2">
+        <v>46104</v>
+      </c>
+      <c r="C47" s="2">
+        <v>46111</v>
+      </c>
+      <c r="D47" t="s">
+        <v>81</v>
+      </c>
+      <c r="U47" s="9"/>
+    </row>
+    <row r="49" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A49" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B49" s="2">
+        <v>46069</v>
+      </c>
+      <c r="C49" s="2">
+        <v>46141</v>
+      </c>
+      <c r="D49" t="s">
+        <v>86</v>
+      </c>
+      <c r="P49" s="17"/>
+      <c r="Q49" s="17"/>
+      <c r="R49" s="17"/>
+      <c r="S49" s="17"/>
+      <c r="T49" s="17"/>
+      <c r="U49" s="17"/>
+      <c r="V49" s="17"/>
+      <c r="W49" s="17"/>
+      <c r="X49" s="17"/>
+      <c r="Y49" s="17"/>
+      <c r="Z49" s="17"/>
+      <c r="AA49" s="17"/>
+    </row>
+    <row r="50" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A50" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B50" s="2">
+        <v>46069</v>
+      </c>
+      <c r="C50" s="2">
+        <v>46076</v>
+      </c>
+      <c r="D50" t="s">
+        <v>81</v>
+      </c>
+      <c r="P50" s="18"/>
+    </row>
+    <row r="51" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A51" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B51" s="2">
+        <v>46076</v>
+      </c>
+      <c r="C51" s="2">
         <v>46083</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B28" s="2">
+      <c r="D51" t="s">
+        <v>81</v>
+      </c>
+      <c r="Q51" s="18"/>
+    </row>
+    <row r="52" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A52" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B52" s="2">
+        <v>46090</v>
+      </c>
+      <c r="C52" s="2">
         <v>46097</v>
       </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B29" s="2">
+      <c r="D52" t="s">
+        <v>81</v>
+      </c>
+      <c r="R52" s="18"/>
+    </row>
+    <row r="53" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A53" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B53" s="2">
+        <v>46111</v>
+      </c>
+      <c r="C53" s="2">
+        <v>46118</v>
+      </c>
+      <c r="D53" t="s">
+        <v>81</v>
+      </c>
+      <c r="S53" s="18"/>
+    </row>
+    <row r="54" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A54" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B54" s="2">
+        <v>46097</v>
+      </c>
+      <c r="C54" s="2">
         <v>46104</v>
       </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" s="3" t="s">
+      <c r="D54" t="s">
+        <v>81</v>
+      </c>
+      <c r="V54" s="18"/>
+    </row>
+    <row r="55" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A55" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B55" s="2">
+        <v>46118</v>
+      </c>
+      <c r="C55" s="2">
+        <v>46125</v>
+      </c>
+      <c r="D55" t="s">
+        <v>81</v>
+      </c>
+      <c r="T55" s="18"/>
+    </row>
+    <row r="56" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A56" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B56" s="2">
+        <v>46125</v>
+      </c>
+      <c r="C56" s="2">
+        <v>46132</v>
+      </c>
+      <c r="D56" t="s">
+        <v>81</v>
+      </c>
+      <c r="W56" s="18"/>
+    </row>
+    <row r="57" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="X57" s="18"/>
+    </row>
+    <row r="58" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A58" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="59" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A59" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B59" s="2">
+        <v>46134</v>
+      </c>
+      <c r="C59" s="2">
+        <v>46134</v>
+      </c>
+      <c r="D59" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="60" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A60" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B60" s="2">
+        <v>46141</v>
+      </c>
+      <c r="C60" s="2">
+        <v>46141</v>
+      </c>
+      <c r="D60" t="s">
+        <v>79</v>
+      </c>
+      <c r="Y60" s="11"/>
+    </row>
+    <row r="61" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="Z61" s="12"/>
+    </row>
+    <row r="62" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A62" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
+    <row r="63" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A63" s="3" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B37" s="2">
+      <c r="B63" s="2">
         <v>46141</v>
       </c>
-      <c r="C37" s="2">
+      <c r="C63" s="2">
         <v>46148</v>
       </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B38" s="2">
+      <c r="D63" t="s">
+        <v>79</v>
+      </c>
+      <c r="Z63" s="10"/>
+      <c r="AA63" s="10"/>
+    </row>
+    <row r="64" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A64" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B64" s="2">
         <v>46149</v>
       </c>
-      <c r="C38" s="2">
+      <c r="C64" s="2">
         <v>46150</v>
       </c>
+      <c r="D64" t="s">
+        <v>79</v>
+      </c>
+      <c r="AA64" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
commit: minor gantt chart fixes
</commit_message>
<xml_diff>
--- a/Documents/Gantt Chart.xlsx
+++ b/Documents/Gantt Chart.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Jerry\Documents\GitHub\Honours-Project-PCG-of-3D-Platformers-\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95219DAA-EE12-42A7-8F9F-FD057ED65CBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04734945-5ED6-4D05-A04F-4B1686D223FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{1119FB18-55D4-4D97-9D7D-B7A1FA1BF5AA}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="91">
   <si>
     <t>Task</t>
   </si>
@@ -303,13 +303,19 @@
   </si>
   <si>
     <t>Player Character Model, Animations, and Refinement</t>
+  </si>
+  <si>
+    <t>29 days</t>
+  </si>
+  <si>
+    <t>10 days</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -328,6 +334,13 @@
     <font>
       <sz val="11"/>
       <color theme="9" tint="-0.249977111117893"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="2" tint="-0.249977111117893"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -419,7 +432,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -443,6 +456,7 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -777,7 +791,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C63CAE2-8401-49FA-BE9B-32E21946B78F}">
-  <dimension ref="A7:AB64"/>
+  <dimension ref="A7:AB65"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="56.42578125" bestFit="1" customWidth="1"/>
@@ -1414,6 +1428,19 @@
       <c r="A43" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="B43" s="2">
+        <v>46083</v>
+      </c>
+      <c r="C43" s="2">
+        <v>46111</v>
+      </c>
+      <c r="D43" t="s">
+        <v>89</v>
+      </c>
+      <c r="R43" s="19"/>
+      <c r="S43" s="19"/>
+      <c r="T43" s="19"/>
+      <c r="U43" s="19"/>
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
@@ -1613,6 +1640,15 @@
       <c r="A58" s="1" t="s">
         <v>39</v>
       </c>
+      <c r="B58" s="2">
+        <v>46134</v>
+      </c>
+      <c r="C58" s="2">
+        <v>46141</v>
+      </c>
+      <c r="D58" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="59" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
@@ -1627,6 +1663,8 @@
       <c r="D59" t="s">
         <v>79</v>
       </c>
+      <c r="Y59" s="8"/>
+      <c r="Z59" s="8"/>
     </row>
     <row r="60" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="s">
@@ -1650,6 +1688,15 @@
       <c r="A62" s="1" t="s">
         <v>21</v>
       </c>
+      <c r="B62" s="2">
+        <v>46141</v>
+      </c>
+      <c r="C62" s="2">
+        <v>46150</v>
+      </c>
+      <c r="D62" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="63" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A63" s="3" t="s">
@@ -1662,10 +1709,10 @@
         <v>46148</v>
       </c>
       <c r="D63" t="s">
-        <v>79</v>
-      </c>
-      <c r="Z63" s="10"/>
-      <c r="AA63" s="10"/>
+        <v>81</v>
+      </c>
+      <c r="Z63" s="8"/>
+      <c r="AA63" s="8"/>
     </row>
     <row r="64" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
@@ -1678,9 +1725,13 @@
         <v>46150</v>
       </c>
       <c r="D64" t="s">
-        <v>79</v>
-      </c>
+        <v>83</v>
+      </c>
+      <c r="Z64" s="10"/>
       <c r="AA64" s="10"/>
+    </row>
+    <row r="65" spans="27:27" x14ac:dyDescent="0.25">
+      <c r="AA65" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
added: small, medium, and large inclines
</commit_message>
<xml_diff>
--- a/Documents/Gantt Chart.xlsx
+++ b/Documents/Gantt Chart.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Jerry\Documents\GitHub\Honours-Project-PCG-of-3D-Platformers-\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04734945-5ED6-4D05-A04F-4B1686D223FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C844198-8537-4B58-A900-023A76FF5F15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{1119FB18-55D4-4D97-9D7D-B7A1FA1BF5AA}"/>
   </bookViews>
@@ -451,12 +451,12 @@
     <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -980,7 +980,7 @@
       <c r="H10" s="8"/>
       <c r="I10" s="8"/>
       <c r="J10" s="8"/>
-      <c r="K10" s="8"/>
+      <c r="K10" s="19"/>
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
@@ -999,7 +999,7 @@
       <c r="H11" s="6"/>
       <c r="I11" s="6"/>
       <c r="J11" s="6"/>
-      <c r="K11" s="6"/>
+      <c r="K11" s="19"/>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="J16" s="7"/>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
         <v>29</v>
       </c>
@@ -1091,7 +1091,7 @@
       </c>
       <c r="J17" s="7"/>
     </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>42</v>
       </c>
@@ -1104,9 +1104,9 @@
       <c r="D18" t="s">
         <v>74</v>
       </c>
-      <c r="H18" s="16"/>
-    </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="H18" s="15"/>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>43</v>
       </c>
@@ -1119,11 +1119,11 @@
       <c r="D19" t="s">
         <v>77</v>
       </c>
-      <c r="G19" s="15"/>
-      <c r="H19" s="15"/>
-      <c r="I19" s="15"/>
-    </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="G19" s="14"/>
+      <c r="H19" s="14"/>
+      <c r="I19" s="14"/>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>45</v>
       </c>
@@ -1139,7 +1139,7 @@
       <c r="I20" s="5"/>
       <c r="J20" s="5"/>
     </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>46</v>
       </c>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="I21" s="5"/>
     </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>47</v>
       </c>
@@ -1169,7 +1169,7 @@
       </c>
       <c r="I22" s="5"/>
     </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>48</v>
       </c>
@@ -1184,7 +1184,7 @@
       </c>
       <c r="J23" s="11"/>
     </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>3</v>
       </c>
@@ -1204,9 +1204,8 @@
       <c r="P25" s="8"/>
       <c r="Q25" s="8"/>
       <c r="R25" s="8"/>
-      <c r="S25" s="14"/>
-    </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>4</v>
       </c>
@@ -1221,7 +1220,7 @@
       </c>
       <c r="L26" s="7"/>
     </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>5</v>
       </c>
@@ -1236,7 +1235,7 @@
       </c>
       <c r="M27" s="7"/>
     </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>88</v>
       </c>
@@ -1251,7 +1250,7 @@
       </c>
       <c r="N28" s="7"/>
     </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>6</v>
       </c>
@@ -1266,7 +1265,7 @@
       </c>
       <c r="N29" s="7"/>
     </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>7</v>
       </c>
@@ -1282,7 +1281,7 @@
       <c r="O30" s="7"/>
       <c r="P30" s="7"/>
     </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>30</v>
       </c>
@@ -1297,9 +1296,8 @@
       </c>
       <c r="P31" s="7"/>
       <c r="Q31" s="7"/>
-      <c r="S31" s="14"/>
-    </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.25">
+    </row>
+    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
         <v>31</v>
       </c>
@@ -1332,7 +1330,6 @@
       <c r="R34" s="8"/>
       <c r="S34" s="8"/>
       <c r="T34" s="8"/>
-      <c r="U34" s="14"/>
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
@@ -1378,7 +1375,6 @@
       <c r="D37" t="s">
         <v>81</v>
       </c>
-      <c r="R37" s="14"/>
       <c r="S37" s="13"/>
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
@@ -1394,7 +1390,6 @@
       <c r="D38" t="s">
         <v>81</v>
       </c>
-      <c r="S38" s="14"/>
       <c r="T38" s="13"/>
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
@@ -1422,7 +1417,6 @@
       <c r="Q41" s="5"/>
       <c r="R41" s="5"/>
       <c r="S41" s="5"/>
-      <c r="T41" s="14"/>
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
@@ -1437,10 +1431,10 @@
       <c r="D43" t="s">
         <v>89</v>
       </c>
-      <c r="R43" s="19"/>
-      <c r="S43" s="19"/>
-      <c r="T43" s="19"/>
-      <c r="U43" s="19"/>
+      <c r="R43" s="18"/>
+      <c r="S43" s="18"/>
+      <c r="T43" s="18"/>
+      <c r="U43" s="18"/>
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
@@ -1515,18 +1509,18 @@
       <c r="D49" t="s">
         <v>86</v>
       </c>
-      <c r="P49" s="17"/>
-      <c r="Q49" s="17"/>
-      <c r="R49" s="17"/>
-      <c r="S49" s="17"/>
-      <c r="T49" s="17"/>
-      <c r="U49" s="17"/>
-      <c r="V49" s="17"/>
-      <c r="W49" s="17"/>
-      <c r="X49" s="17"/>
-      <c r="Y49" s="17"/>
-      <c r="Z49" s="17"/>
-      <c r="AA49" s="17"/>
+      <c r="P49" s="16"/>
+      <c r="Q49" s="16"/>
+      <c r="R49" s="16"/>
+      <c r="S49" s="16"/>
+      <c r="T49" s="16"/>
+      <c r="U49" s="16"/>
+      <c r="V49" s="16"/>
+      <c r="W49" s="16"/>
+      <c r="X49" s="16"/>
+      <c r="Y49" s="16"/>
+      <c r="Z49" s="16"/>
+      <c r="AA49" s="16"/>
     </row>
     <row r="50" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
@@ -1541,7 +1535,7 @@
       <c r="D50" t="s">
         <v>81</v>
       </c>
-      <c r="P50" s="18"/>
+      <c r="P50" s="17"/>
     </row>
     <row r="51" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
@@ -1556,7 +1550,7 @@
       <c r="D51" t="s">
         <v>81</v>
       </c>
-      <c r="Q51" s="18"/>
+      <c r="Q51" s="17"/>
     </row>
     <row r="52" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
@@ -1571,7 +1565,7 @@
       <c r="D52" t="s">
         <v>81</v>
       </c>
-      <c r="R52" s="18"/>
+      <c r="R52" s="17"/>
     </row>
     <row r="53" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
@@ -1586,7 +1580,7 @@
       <c r="D53" t="s">
         <v>81</v>
       </c>
-      <c r="S53" s="18"/>
+      <c r="S53" s="17"/>
     </row>
     <row r="54" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
@@ -1601,7 +1595,7 @@
       <c r="D54" t="s">
         <v>81</v>
       </c>
-      <c r="V54" s="18"/>
+      <c r="V54" s="17"/>
     </row>
     <row r="55" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
@@ -1616,7 +1610,7 @@
       <c r="D55" t="s">
         <v>81</v>
       </c>
-      <c r="T55" s="18"/>
+      <c r="T55" s="17"/>
     </row>
     <row r="56" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
@@ -1631,10 +1625,10 @@
       <c r="D56" t="s">
         <v>81</v>
       </c>
-      <c r="W56" s="18"/>
+      <c r="W56" s="17"/>
     </row>
     <row r="57" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="X57" s="18"/>
+      <c r="X57" s="17"/>
     </row>
     <row r="58" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">

</xml_diff>